<commit_message>
arreglo de errores ERR-14....
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/_verificacion_2026-10-17/Matriz de verificación cruzada.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/_verificacion_2026-10-17/Matriz de verificación cruzada.xlsx
@@ -13722,12 +13722,12 @@
       </c>
       <c r="H214" s="2" t="inlineStr">
         <is>
-          <t>Informe TEC: el índice anuncia "Presupuesto de Infraestructura..." pero la sección no existe</t>
+          <t>Informe TEC: sección «Presupuesto de Infraestructura y Herramientas a Utilizar» presente entre «Tarifas» y «Resumen Financiero»; el índice enlaza a ella (marcador _9m3x90b8fdyy). Total $1.496.400 sin cambios.</t>
         </is>
       </c>
       <c r="I214" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
@@ -13737,12 +13737,12 @@
       </c>
       <c r="K214" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="L214" s="2" t="inlineStr">
         <is>
-          <t>Incorporado a Cambios Pendientes el 17/10/2026</t>
+          <t>Corregido el 18/10/2026: sección creada con costos conocidos ($0 en herramientas, PayPal sandbox, Firebase, Maps, jsReport, Mindicador) y pendientes marcados (mensajería, hosting, tiendas). Causa raíz confirmada: sección inexistente. Archivo: Informe TEC.docx. Limitación: páginas del índice sin actualizar (hacerlo en Word); no abierto en Word para revisión visual.</t>
         </is>
       </c>
     </row>
@@ -13784,12 +13784,12 @@
       </c>
       <c r="H215" s="2" t="inlineStr">
         <is>
-          <t>Horas hombre: F10:F36 siguen con =MULTIPLY(...) y totales "88h" / "$1.032.000CLP" escritos a mano</t>
+          <t>Horas hombre: F10:F36 = E*C (sin MULTIPLY); C38 =SUM(C10:C36) = 88 h; F38 =SUM(F10:F36) = $1.032.000. Comprobado por recálculo en Python sobre el detalle.</t>
         </is>
       </c>
       <c r="I215" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
@@ -13799,12 +13799,12 @@
       </c>
       <c r="K215" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="L215" s="2" t="inlineStr">
         <is>
-          <t>Incorporado a Cambios Pendientes el 17/10/2026</t>
+          <t>Corregido el 18/10/2026: fórmulas =E*C y totales =SUM. Causa raíz confirmada: MULTIPLY no existe en Excel y los totales estaban escritos a mano. Archivo: Horas hombre en relación a Tareas.xlsx. Limitación: no abierto en Excel para ver el recálculo.</t>
         </is>
       </c>
     </row>
@@ -13846,12 +13846,12 @@
       </c>
       <c r="H216" s="2" t="inlineStr">
         <is>
-          <t>Horas hombre: resumen sigue Gabriel 29 h/$348.000 y Alonso 12 h/$120.000 (el detalle da Gabriel 12 h y Alonso 29 h)</t>
+          <t>Horas hombre: resumen con SUMIF: Gabriel 12 h/$120.000; Diego 47 h/$564.000; Alonso 29 h/$348.000 (criterio 'Alonso*'). Comprobado por recálculo: coincide con el detalle.</t>
         </is>
       </c>
       <c r="I216" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
@@ -13861,12 +13861,12 @@
       </c>
       <c r="K216" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="L216" s="2" t="inlineStr">
         <is>
-          <t>Incorporado a Cambios Pendientes el 17/10/2026</t>
+          <t>Corregido el 18/10/2026: resumen por responsable con SUMIF sobre la columna D. Causa raíz confirmada: valores fijos intercambiados entre Gabriel y Alonso. Riesgo evitado: «Alonso Gonzalez» (sin tilde) en el detalle; con coincidencia exacta el SUMIF daría 0. Archivo: Horas hombre en relación a Tareas.xlsx.</t>
         </is>
       </c>
     </row>
@@ -17379,12 +17379,12 @@
       <c r="F74" s="2" t="n"/>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Informe TEC: el índice anuncia "Presupuesto de Infraestructura..." pero la sección no existe</t>
+          <t>Informe TEC: sección «Presupuesto de Infraestructura y Herramientas a Utilizar» presente entre «Tarifas» y «Resumen Financiero»; el índice enlaza a ella (marcador _9m3x90b8fdyy). Total $1.496.400 sin cambios.</t>
         </is>
       </c>
     </row>
@@ -17455,12 +17455,12 @@
       <c r="F76" s="2" t="n"/>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Horas hombre: F10:F36 siguen con =MULTIPLY(...) y totales "88h" / "$1.032.000CLP" escritos a mano</t>
+          <t>Horas hombre: F10:F36 = E*C (sin MULTIPLY); C38 =SUM(C10:C36) = 88 h; F38 =SUM(F10:F36) = $1.032.000. Comprobado por recálculo en Python sobre el detalle.</t>
         </is>
       </c>
     </row>
@@ -17493,12 +17493,12 @@
       <c r="F77" s="2" t="n"/>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Horas hombre: resumen sigue Gabriel 29 h/$348.000 y Alonso 12 h/$120.000 (el detalle da Gabriel 12 h y Alonso 29 h)</t>
+          <t>Horas hombre: resumen con SUMIF: Gabriel 12 h/$120.000; Diego 47 h/$564.000; Alonso 29 h/$348.000 (criterio 'Alonso*'). Comprobado por recálculo: coincide con el detalle.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
arreglo de [ERR-12] Errores de planificación (sprints, fechas y backlog)
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/_verificacion_2026-10-17/Matriz de verificación cruzada.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/_verificacion_2026-10-17/Matriz de verificación cruzada.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L225"/>
+  <dimension ref="A1:L232"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="3"/>
@@ -12229,7 +12229,7 @@
       </c>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>Ausente</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="H190" s="2" t="inlineStr">
@@ -12239,22 +12239,22 @@
       </c>
       <c r="I190" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="K190" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="L190" s="2" t="inlineStr">
         <is>
-          <t>Mantener en Cambios Pendientes</t>
+          <t>Resuelto el 18/10/2026. Hoja de ruta §7: horizonte de 5 semanas (antes 7). Verificado en el archivo.</t>
         </is>
       </c>
     </row>
@@ -12353,7 +12353,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>Ausente</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -12363,22 +12363,22 @@
       </c>
       <c r="I192" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="L192" s="2" t="inlineStr">
         <is>
-          <t>Mantener en Cambios Pendientes</t>
+          <t>Resuelto el 18/10/2026. Hoja de ruta §7: nota de fechas añadida con el texto aprobado. Verificado en el archivo.</t>
         </is>
       </c>
     </row>
@@ -12415,7 +12415,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>Ausente</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -12425,22 +12425,22 @@
       </c>
       <c r="I193" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
         <is>
-          <t>Mantener en Cambios Pendientes</t>
+          <t>Resuelto el 18/10/2026. Hoja de ruta §6: DoD única de 8 ítems; eliminada la lista de 6. Verificado en el archivo.</t>
         </is>
       </c>
     </row>
@@ -12477,7 +12477,7 @@
       </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t>Ausente</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="H194" s="2" t="inlineStr">
@@ -12487,22 +12487,22 @@
       </c>
       <c r="I194" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="L194" s="2" t="inlineStr">
         <is>
-          <t>Mantener en Cambios Pendientes</t>
+          <t>Resuelto el 18/10/2026. Sprint-fase1: F1-01…F1-11 cambiados a TD-01…TD-11. Verificado en el archivo.</t>
         </is>
       </c>
     </row>
@@ -12626,7 +12626,7 @@
       </c>
       <c r="L196" s="2" t="inlineStr">
         <is>
-          <t>Incorporado a Cambios Pendientes el 17/10/2026</t>
+          <t>Pendiente: texto de la nota de planificación por HU en el ERS sin aprobar (decisión 18/10/2026).</t>
         </is>
       </c>
     </row>
@@ -12663,7 +12663,7 @@
       </c>
       <c r="G197" s="2" t="inlineStr">
         <is>
-          <t>Ausente</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="H197" s="2" t="inlineStr">
@@ -12673,22 +12673,22 @@
       </c>
       <c r="I197" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="L197" s="2" t="inlineStr">
         <is>
-          <t>Mantener en Cambios Pendientes</t>
+          <t>Resuelto el 18/10/2026. Product Backlog §3 y §7: cierre de Fase 1 el 14 de septiembre. Verificado en el archivo.</t>
         </is>
       </c>
     </row>
@@ -12725,7 +12725,7 @@
       </c>
       <c r="G198" s="2" t="inlineStr">
         <is>
-          <t>Ausente</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="H198" s="2" t="inlineStr">
@@ -12735,22 +12735,22 @@
       </c>
       <c r="I198" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="L198" s="2" t="inlineStr">
         <is>
-          <t>Incorporado a Cambios Pendientes el 17/10/2026</t>
+          <t>Resuelto el 18/10/2026. Product Backlog §7: cadencia de tres Sprints de una semana y el Sprint 4 de dos. Verificado en el archivo.</t>
         </is>
       </c>
     </row>
@@ -12812,7 +12812,7 @@
       </c>
       <c r="L199" s="2" t="inlineStr">
         <is>
-          <t>Incorporado a Cambios Pendientes el 17/10/2026</t>
+          <t>Pendiente: TD-12 en el Sprint 4 del Backlog; decisión diferida por el usuario (18/10/2026).</t>
         </is>
       </c>
     </row>
@@ -12849,7 +12849,7 @@
       </c>
       <c r="G200" s="2" t="inlineStr">
         <is>
-          <t>Ausente</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="H200" s="2" t="inlineStr">
@@ -12859,22 +12859,22 @@
       </c>
       <c r="I200" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="L200" s="2" t="inlineStr">
         <is>
-          <t>Mantener en Cambios Pendientes</t>
+          <t>Resuelto el 18/10/2026. Product Backlog §7: DoD de 6 ítems sustituida por remisión a la DoD única (Hoja §6). Verificado.</t>
         </is>
       </c>
     </row>
@@ -12911,7 +12911,7 @@
       </c>
       <c r="G201" s="2" t="inlineStr">
         <is>
-          <t>Ausente</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="H201" s="2" t="inlineStr">
@@ -12921,22 +12921,22 @@
       </c>
       <c r="I201" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="L201" s="2" t="inlineStr">
         <is>
-          <t>Incorporado a Cambios Pendientes el 17/10/2026</t>
+          <t>Resuelto el 18/10/2026. Product Backlog §8: columna Sprint renumerada +4 (Sprint 5 a 15). Resuelto con observación: 1.2.3 no documenta Sprints 8 a 15.</t>
         </is>
       </c>
     </row>
@@ -12973,7 +12973,7 @@
       </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
-          <t>Ausente</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="H202" s="2" t="inlineStr">
@@ -12983,22 +12983,22 @@
       </c>
       <c r="I202" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="L202" s="2" t="inlineStr">
         <is>
-          <t>Incorporado a Cambios Pendientes el 17/10/2026</t>
+          <t>Resuelto el 18/10/2026. Tabla Maestra, Maestro y Tareas F1: dependencias F1-xx cambiadas a TD-xx (solo filas TD). Verificado.</t>
         </is>
       </c>
     </row>
@@ -13035,7 +13035,7 @@
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t>Ausente</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="H203" s="2" t="inlineStr">
@@ -13045,22 +13045,22 @@
       </c>
       <c r="I203" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="L203" s="2" t="inlineStr">
         <is>
-          <t>Incorporado a Cambios Pendientes el 17/10/2026</t>
+          <t>Resuelto el 18/10/2026. Tabla Maestra, Tareas F1: TD-05 y TD-06 con prioridad Media (como en Maestro); IDs TD-xx. Verificado.</t>
         </is>
       </c>
     </row>
@@ -13127,448 +13127,448 @@
       </c>
     </row>
     <row r="205" ht="45" customHeight="1">
-      <c r="A205" s="2" t="inlineStr">
-        <is>
-          <t>[ERR-13.01]</t>
-        </is>
-      </c>
-      <c r="B205" s="2" t="inlineStr">
-        <is>
-          <t>AUDIT-005</t>
-        </is>
-      </c>
-      <c r="C205" s="2" t="inlineStr">
-        <is>
-          <t>ERR-13 Errores de roles y responsabilidades</t>
-        </is>
-      </c>
-      <c r="D205" s="2" t="inlineStr">
-        <is>
-          <t>Acta de constitución: La Lista de Interesados conservaba nombres de la plantilla en lugar del interesado real (Julio Tapia, Product Owner).</t>
-        </is>
-      </c>
-      <c r="E205" s="2" t="inlineStr">
-        <is>
-          <t>Fuente B: bloque ERR-13 · Fuente A: AUDIT-005, párrafo P11 (Acta de Constitución)</t>
-        </is>
-      </c>
-      <c r="F205" s="2" t="inlineStr">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>[ERR-12.18]</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Nuevo (sin AUDIT)</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>ERR-12 Errores de planificación (sprints, fechas y backlog)</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Product Backlog §7: periodos de Sprints 1–3 (10–16, 17–23, 24–30 ago) no coincidían con la Hoja de ruta.</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>2.1.1 PRODUCT BACKLOG §7</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Ausente (hallazgo nuevo)</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>Hoja de ruta y Sprint-fase1: 10–14, 17–21 y 24–28 ago</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>Resuelto el 18/10/2026. Periodos alineados con la Hoja de ruta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206" ht="45" customHeight="1">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>[ERR-12.19]</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Nuevo (sin AUDIT)</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>ERR-12 Errores de planificación (sprints, fechas y backlog)</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Sprint-fase1: hito académico del Sprint 4 "jueves 4"; el 4/9/2026 es viernes.</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>1.2.2 Sprint-fase1</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Ausente (hallazgo nuevo)</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>Sprint-fase1: "viernes 4 a las 1:40"</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>Resuelto el 18/10/2026. Día corregido a viernes, según decisión del usuario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" ht="45" customHeight="1">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>[ERR-12.20]</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Nuevo (sin AUDIT)</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>ERR-12 Errores de planificación (sprints, fechas y backlog)</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Trello.json: listas "Cierre Sprint 4" con fechas 4/9 (cerrada) y 14/9 (abierta).</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Trello.json (referencia)</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Ausente (hallazgo nuevo)</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
         <is>
           <t>Ausente</t>
         </is>
       </c>
-      <c r="G205" s="2" t="inlineStr">
-        <is>
-          <t>Presente</t>
-        </is>
-      </c>
-      <c r="H205" s="2" t="inlineStr">
-        <is>
-          <t>Acta: Lista de Interesados = Julio Tapia (Product Owner)</t>
-        </is>
-      </c>
-      <c r="I205" s="3" t="inlineStr">
-        <is>
-          <t>Verificado</t>
-        </is>
-      </c>
-      <c r="J205" s="2" t="inlineStr">
-        <is>
-          <t>verde parcial</t>
-        </is>
-      </c>
-      <c r="K205" s="2" t="inlineStr">
-        <is>
-          <t>verde parcial</t>
-        </is>
-      </c>
-      <c r="L205" s="2" t="inlineStr">
-        <is>
-          <t>Mantener (verde correcto)</t>
-        </is>
-      </c>
-    </row>
-    <row r="206" ht="45" customHeight="1">
-      <c r="A206" s="2" t="inlineStr">
-        <is>
-          <t>[ERR-13.02]</t>
-        </is>
-      </c>
-      <c r="B206" s="2" t="inlineStr">
-        <is>
-          <t>AUDIT-006</t>
-        </is>
-      </c>
-      <c r="C206" s="2" t="inlineStr">
-        <is>
-          <t>ERR-13 Errores de roles y responsabilidades</t>
-        </is>
-      </c>
-      <c r="D206" s="2" t="inlineStr">
-        <is>
-          <t>1.2.1 Hoja de ruta del proyecto: Alineación con la Capacidad Real mencionaba 'dos Developers' en lugar de tres.</t>
-        </is>
-      </c>
-      <c r="E206" s="2" t="inlineStr">
-        <is>
-          <t>Fuente B: bloque ERR-13 · Fuente A: AUDIT-006, párrafo P14 (1.2.1 Hoja de ruta del proyecto)</t>
-        </is>
-      </c>
-      <c r="F206" s="2" t="inlineStr">
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>Documentos y Sprint-fase1: cierre 14/9</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>Pendiente (Trello)</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>Pendiente desde 18/10/2026. No se modifica Trello.json; decisión del equipo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" ht="45" customHeight="1">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>[ERR-12.21]</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Nuevo (sin AUDIT)</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>ERR-12 Errores de planificación (sprints, fechas y backlog)</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Trello.json: tarjeta "Sprint Review" del Sprint 4 con fecha 3/9, en la lista de cierre 14/9.</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Trello.json (referencia)</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Ausente (hallazgo nuevo)</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
         <is>
           <t>Ausente</t>
         </is>
       </c>
-      <c r="G206" s="2" t="inlineStr">
-        <is>
-          <t>Presente</t>
-        </is>
-      </c>
-      <c r="H206" s="2" t="inlineStr">
-        <is>
-          <t>Hoja de ruta §7: "equipo de tres Developers"</t>
-        </is>
-      </c>
-      <c r="I206" s="3" t="inlineStr">
-        <is>
-          <t>Verificado</t>
-        </is>
-      </c>
-      <c r="J206" s="2" t="inlineStr">
-        <is>
-          <t>verde parcial</t>
-        </is>
-      </c>
-      <c r="K206" s="2" t="inlineStr">
-        <is>
-          <t>verde parcial</t>
-        </is>
-      </c>
-      <c r="L206" s="2" t="inlineStr">
-        <is>
-          <t>Mantener (verde correcto)</t>
-        </is>
-      </c>
-    </row>
-    <row r="207" ht="45" customHeight="1">
-      <c r="A207" s="2" t="inlineStr">
-        <is>
-          <t>[ERR-13.03]</t>
-        </is>
-      </c>
-      <c r="B207" s="2" t="inlineStr">
-        <is>
-          <t>AUDIT-024</t>
-        </is>
-      </c>
-      <c r="C207" s="2" t="inlineStr">
-        <is>
-          <t>ERR-13 Errores de roles y responsabilidades</t>
-        </is>
-      </c>
-      <c r="D207" s="2" t="inlineStr">
-        <is>
-          <t>1.2.1 Hoja de ruta del proyecto: La sección Trabajo en Paralelo seguía mencionando 'dos Developers' cuando el equipo tiene tres.</t>
-        </is>
-      </c>
-      <c r="E207" s="2" t="inlineStr">
-        <is>
-          <t>Fuente B: bloque ERR-13 · Fuente A: AUDIT-024, párrafo P66 (1.2.1 Hoja de ruta del proyecto.docx (1.2))</t>
-        </is>
-      </c>
-      <c r="F207" s="2" t="inlineStr">
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>Sprint-fase1: Review del Sprint 4 registrada el 14/9</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>Pendiente (Trello)</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>Pendiente desde 18/10/2026. Usuario confirmó 14/9; Trello sin modificar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209" ht="45" customHeight="1">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>[ERR-12.22]</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Nuevo (sin AUDIT)</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>ERR-12 Errores de planificación (sprints, fechas y backlog)</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Trello.json: listas duplicadas (Cierre Sprint 3; Daily sprint 2, 3 y 4; Sprint 6).</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Trello.json (referencia)</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Ausente (hallazgo nuevo)</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
         <is>
           <t>Ausente</t>
         </is>
       </c>
-      <c r="G207" s="2" t="inlineStr">
-        <is>
-          <t>Presente</t>
-        </is>
-      </c>
-      <c r="H207" s="2" t="inlineStr">
-        <is>
-          <t>Hoja de ruta: "dos de los tres Developers"</t>
-        </is>
-      </c>
-      <c r="I207" s="3" t="inlineStr">
-        <is>
-          <t>Verificado</t>
-        </is>
-      </c>
-      <c r="J207" s="2" t="inlineStr">
-        <is>
-          <t>verde</t>
-        </is>
-      </c>
-      <c r="K207" s="2" t="inlineStr">
-        <is>
-          <t>verde</t>
-        </is>
-      </c>
-      <c r="L207" s="2" t="inlineStr">
-        <is>
-          <t>Mantener (verde correcto)</t>
-        </is>
-      </c>
-    </row>
-    <row r="208" ht="45" customHeight="1">
-      <c r="A208" s="2" t="inlineStr">
-        <is>
-          <t>[ERR-13.04]</t>
-        </is>
-      </c>
-      <c r="B208" s="2" t="inlineStr">
-        <is>
-          <t>AUDIT-069</t>
-        </is>
-      </c>
-      <c r="C208" s="2" t="inlineStr">
-        <is>
-          <t>ERR-13 Errores de roles y responsabilidades</t>
-        </is>
-      </c>
-      <c r="D208" s="2" t="inlineStr">
-        <is>
-          <t>Matriz RACI: La misma persona era Responsable (R) y Aprobador (A) en Desarrollo de la Aplicación de Escritorio.</t>
-        </is>
-      </c>
-      <c r="E208" s="2" t="inlineStr">
-        <is>
-          <t>Fuente B: bloque ERR-13 · Fuente A: AUDIT-069, párrafo P251 (Matriz RACI.xlsx (1.5))</t>
-        </is>
-      </c>
-      <c r="F208" s="2" t="inlineStr">
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>Lista de Trello por nombre y estado</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>Pendiente (Trello)</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>Pendiente desde 18/10/2026. No se modifica Trello.json.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" ht="45" customHeight="1">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>[ERR-12.23]</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Nuevo (sin AUDIT)</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>ERR-12 Errores de planificación (sprints, fechas y backlog)</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Trello.json: 23 listas "Sprint 6 a 28 - 10/8/2026" cerradas, con fechas que no corresponden.</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Trello.json (referencia)</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Ausente (hallazgo nuevo)</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
         <is>
           <t>Ausente</t>
         </is>
       </c>
-      <c r="G208" s="2" t="inlineStr">
-        <is>
-          <t>Presente</t>
-        </is>
-      </c>
-      <c r="H208" s="2" t="inlineStr">
-        <is>
-          <t>Matriz RACI: filas 10, 11, 2-3 y 14 según lo indicado</t>
-        </is>
-      </c>
-      <c r="I208" s="3" t="inlineStr">
-        <is>
-          <t>Verificado</t>
-        </is>
-      </c>
-      <c r="J208" s="2" t="inlineStr">
-        <is>
-          <t>verde parcial</t>
-        </is>
-      </c>
-      <c r="K208" s="2" t="inlineStr">
-        <is>
-          <t>verde parcial</t>
-        </is>
-      </c>
-      <c r="L208" s="2" t="inlineStr">
-        <is>
-          <t>Mantener (verde correcto)</t>
-        </is>
-      </c>
-    </row>
-    <row r="209" ht="45" customHeight="1">
-      <c r="A209" s="2" t="inlineStr">
-        <is>
-          <t>[ERR-13.05]</t>
-        </is>
-      </c>
-      <c r="B209" s="2" t="inlineStr">
-        <is>
-          <t>AUDIT-070</t>
-        </is>
-      </c>
-      <c r="C209" s="2" t="inlineStr">
-        <is>
-          <t>ERR-13 Errores de roles y responsabilidades</t>
-        </is>
-      </c>
-      <c r="D209" s="2" t="inlineStr">
-        <is>
-          <t>Matriz RACI: La misma persona era R y A en Testing QA, y el Product Owner solo figuraba como Informado.</t>
-        </is>
-      </c>
-      <c r="E209" s="2" t="inlineStr">
-        <is>
-          <t>Fuente B: bloque ERR-13 · Fuente A: AUDIT-070, párrafo P255 (Matriz RACI.xlsx (1.5))</t>
-        </is>
-      </c>
-      <c r="F209" s="2" t="inlineStr">
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>Lista de Trello por nombre y estado</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>Pendiente (Trello)</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>Pendiente desde 18/10/2026. No se modifica Trello.json.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" ht="45" customHeight="1">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>[ERR-12.24]</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Nuevo (sin AUDIT)</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>ERR-12 Errores de planificación (sprints, fechas y backlog)</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Trello.json: "Cierre Sprint 7 - /10/2026" sin día; "Sprint 7 - 12/10/2026" abierta.</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Trello.json (referencia)</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Ausente (hallazgo nuevo)</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
         <is>
           <t>Ausente</t>
         </is>
       </c>
-      <c r="G209" s="2" t="inlineStr">
-        <is>
-          <t>Presente</t>
-        </is>
-      </c>
-      <c r="H209" s="2" t="inlineStr">
-        <is>
-          <t>Matriz RACI: filas 10, 11, 2-3 y 14 según lo indicado</t>
-        </is>
-      </c>
-      <c r="I209" s="3" t="inlineStr">
-        <is>
-          <t>Verificado</t>
-        </is>
-      </c>
-      <c r="J209" s="2" t="inlineStr">
-        <is>
-          <t>verde parcial</t>
-        </is>
-      </c>
-      <c r="K209" s="2" t="inlineStr">
-        <is>
-          <t>verde parcial</t>
-        </is>
-      </c>
-      <c r="L209" s="2" t="inlineStr">
-        <is>
-          <t>Mantener (verde correcto)</t>
-        </is>
-      </c>
-    </row>
-    <row r="210" ht="45" customHeight="1">
-      <c r="A210" s="2" t="inlineStr">
-        <is>
-          <t>[ERR-13.06]</t>
-        </is>
-      </c>
-      <c r="B210" s="2" t="inlineStr">
-        <is>
-          <t>AUDIT-071</t>
-        </is>
-      </c>
-      <c r="C210" s="2" t="inlineStr">
-        <is>
-          <t>ERR-13 Errores de roles y responsabilidades</t>
-        </is>
-      </c>
-      <c r="D210" s="2" t="inlineStr">
-        <is>
-          <t>Matriz RACI: El Product Owner figuraba solo como Informado, incluso en Definición de requisitos.</t>
-        </is>
-      </c>
-      <c r="E210" s="2" t="inlineStr">
-        <is>
-          <t>Fuente B: bloque ERR-13 · Fuente A: AUDIT-071, párrafo P259 (Matriz RACI.xlsx (1.5))</t>
-        </is>
-      </c>
-      <c r="F210" s="2" t="inlineStr">
-        <is>
-          <t>Ausente</t>
-        </is>
-      </c>
-      <c r="G210" s="2" t="inlineStr">
-        <is>
-          <t>Presente</t>
-        </is>
-      </c>
-      <c r="H210" s="2" t="inlineStr">
-        <is>
-          <t>Matriz RACI: filas 10, 11, 2-3 y 14 según lo indicado</t>
-        </is>
-      </c>
-      <c r="I210" s="3" t="inlineStr">
-        <is>
-          <t>Verificado</t>
-        </is>
-      </c>
-      <c r="J210" s="2" t="inlineStr">
-        <is>
-          <t>verde parcial</t>
-        </is>
-      </c>
-      <c r="K210" s="2" t="inlineStr">
-        <is>
-          <t>verde parcial</t>
-        </is>
-      </c>
-      <c r="L210" s="2" t="inlineStr">
-        <is>
-          <t>Mantener (verde correcto)</t>
-        </is>
-      </c>
-    </row>
-    <row r="211" ht="45" customHeight="1">
-      <c r="A211" s="2" t="inlineStr">
-        <is>
-          <t>[ERR-13.07]</t>
-        </is>
-      </c>
-      <c r="B211" s="2" t="inlineStr">
-        <is>
-          <t>AUDIT-072</t>
-        </is>
-      </c>
-      <c r="C211" s="2" t="inlineStr">
-        <is>
-          <t>ERR-13 Errores de roles y responsabilidades</t>
-        </is>
-      </c>
-      <c r="D211" s="2" t="inlineStr">
-        <is>
-          <t>Matriz RACI: Faltaba la actividad 'Aceptación de incrementos (Sprint Review)' exigida por el Plan de pruebas.</t>
-        </is>
-      </c>
-      <c r="E211" s="2" t="inlineStr">
-        <is>
-          <t>Fuente B: bloque ERR-13 · Fuente A: AUDIT-072, párrafo P263 (Matriz RACI.xlsx (1.5))</t>
-        </is>
-      </c>
-      <c r="F211" s="2" t="inlineStr">
-        <is>
-          <t>Ausente</t>
-        </is>
-      </c>
-      <c r="G211" s="2" t="inlineStr">
-        <is>
-          <t>Presente</t>
-        </is>
-      </c>
-      <c r="H211" s="2" t="inlineStr">
-        <is>
-          <t>Matriz RACI: filas 10, 11, 2-3 y 14 según lo indicado</t>
-        </is>
-      </c>
-      <c r="I211" s="3" t="inlineStr">
-        <is>
-          <t>Verificado</t>
-        </is>
-      </c>
-      <c r="J211" s="2" t="inlineStr">
-        <is>
-          <t>verde parcial</t>
-        </is>
-      </c>
-      <c r="K211" s="2" t="inlineStr">
-        <is>
-          <t>verde parcial</t>
-        </is>
-      </c>
-      <c r="L211" s="2" t="inlineStr">
-        <is>
-          <t>Mantener (verde correcto)</t>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>Lista de Trello por nombre</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>Pendiente (Trello)</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>Pendiente desde 18/10/2026. No se modifica Trello.json.</t>
         </is>
       </c>
     </row>
     <row r="212" ht="45" customHeight="1">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>[ERR-13.08]</t>
+          <t>[ERR-13.01]</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
         <is>
-          <t>AUDIT-112</t>
+          <t>AUDIT-005</t>
         </is>
       </c>
       <c r="C212" s="2" t="inlineStr">
@@ -13578,12 +13578,12 @@
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
-          <t>2.1.1 PRODUCT BACKLOG: Se mencionaban 'dos Developers' cuando el equipo tiene tres integrantes con tareas de desarrollo.</t>
+          <t>Acta de constitución: La Lista de Interesados conservaba nombres de la plantilla en lugar del interesado real (Julio Tapia, Product Owner).</t>
         </is>
       </c>
       <c r="E212" s="2" t="inlineStr">
         <is>
-          <t>Fuente B: bloque ERR-13 · Fuente A: AUDIT-112, párrafo P426 (2.1.1 PRODUCT BACKLOG.docx (2.1))</t>
+          <t>Fuente B: bloque ERR-13 · Fuente A: AUDIT-005, párrafo P11 (Acta de Constitución)</t>
         </is>
       </c>
       <c r="F212" s="2" t="inlineStr">
@@ -13598,7 +13598,7 @@
       </c>
       <c r="H212" s="2" t="inlineStr">
         <is>
-          <t>Product Backlog §10: "tres Developers"</t>
+          <t>Acta: Lista de Interesados = Julio Tapia (Product Owner)</t>
         </is>
       </c>
       <c r="I212" s="3" t="inlineStr">
@@ -13625,12 +13625,12 @@
     <row r="213" ht="45" customHeight="1">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>[ERR-13.09]</t>
+          <t>[ERR-13.02]</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
         <is>
-          <t>AUDIT-P09</t>
+          <t>AUDIT-006</t>
         </is>
       </c>
       <c r="C213" s="2" t="inlineStr">
@@ -13640,99 +13640,99 @@
       </c>
       <c r="D213" s="2" t="inlineStr">
         <is>
-          <t>[Pendiente] Cambios Pendientes: El rebalanceo de la carga de Alonso (BD, web y móvil) en la RACI sigue sin resolverse.</t>
+          <t>1.2.1 Hoja de ruta del proyecto: Alineación con la Capacidad Real mencionaba 'dos Developers' en lugar de tres.</t>
         </is>
       </c>
       <c r="E213" s="2" t="inlineStr">
         <is>
-          <t>Fuente B: bloque ERR-13</t>
+          <t>Fuente B: bloque ERR-13 · Fuente A: AUDIT-006, párrafo P14 (1.2.1 Hoja de ruta del proyecto)</t>
         </is>
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
+          <t>Ausente</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="inlineStr">
+        <is>
           <t>Presente</t>
         </is>
       </c>
-      <c r="G213" s="2" t="inlineStr">
-        <is>
-          <t>Ausente</t>
-        </is>
-      </c>
       <c r="H213" s="2" t="inlineStr">
         <is>
-          <t>Ítem de Cambios Pendientes</t>
-        </is>
-      </c>
-      <c r="I213" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente (AUDIT-P09)</t>
+          <t>Hoja de ruta §7: "equipo de tres Developers"</t>
+        </is>
+      </c>
+      <c r="I213" s="3" t="inlineStr">
+        <is>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde parcial</t>
         </is>
       </c>
       <c r="K213" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde parcial</t>
         </is>
       </c>
       <c r="L213" s="2" t="inlineStr">
         <is>
-          <t>Mantener en Cambios Pendientes</t>
+          <t>Mantener (verde correcto)</t>
         </is>
       </c>
     </row>
     <row r="214" ht="45" customHeight="1">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>[ERR-14.01]</t>
+          <t>[ERR-13.03]</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>AUDIT-073</t>
+          <t>AUDIT-024</t>
         </is>
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>ERR-14 Errores de presupuesto y cálculo</t>
+          <t>ERR-13 Errores de roles y responsabilidades</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
         <is>
-          <t>Informe TEC: El índice anunciaba la sección de Presupuesto de Infraestructura, pero no existía (faltaban costos de SMS, hosting, Maps y tiendas).</t>
+          <t>1.2.1 Hoja de ruta del proyecto: La sección Trabajo en Paralelo seguía mencionando 'dos Developers' cuando el equipo tiene tres.</t>
         </is>
       </c>
       <c r="E214" s="2" t="inlineStr">
         <is>
-          <t>Fuente B: bloque ERR-14 · Fuente A: AUDIT-073, párrafo P268 (Informe TEC.docx (1.6))</t>
+          <t>Fuente B: bloque ERR-13 · Fuente A: AUDIT-024, párrafo P66 (1.2.1 Hoja de ruta del proyecto.docx (1.2))</t>
         </is>
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>Ausente (incorporado el 17/10/2026)</t>
+          <t>Ausente</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
         <is>
-          <t>Ausente</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="H214" s="2" t="inlineStr">
         <is>
-          <t>Informe TEC: sección «Presupuesto de Infraestructura y Herramientas a Utilizar» presente entre «Tarifas» y «Resumen Financiero»; el índice enlaza a ella (marcador _9m3x90b8fdyy). Total $1.496.400 sin cambios.</t>
-        </is>
-      </c>
-      <c r="I214" s="4" t="inlineStr">
+          <t>Hoja de ruta: "dos de los tres Developers"</t>
+        </is>
+      </c>
+      <c r="I214" s="3" t="inlineStr">
         <is>
           <t>Verificado</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="K214" s="2" t="inlineStr">
@@ -13742,235 +13742,235 @@
       </c>
       <c r="L214" s="2" t="inlineStr">
         <is>
-          <t>Corregido el 18/10/2026: sección creada con costos conocidos ($0 en herramientas, PayPal sandbox, Firebase, Maps, jsReport, Mindicador) y pendientes marcados (mensajería, hosting, tiendas). Causa raíz confirmada: sección inexistente. Archivo: Informe TEC.docx. Limitación: páginas del índice sin actualizar (hacerlo en Word); no abierto en Word para revisión visual.</t>
+          <t>Mantener (verde correcto)</t>
         </is>
       </c>
     </row>
     <row r="215" ht="45" customHeight="1">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>[ERR-14.02]</t>
+          <t>[ERR-13.04]</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
         <is>
-          <t>AUDIT-075</t>
+          <t>AUDIT-069</t>
         </is>
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>ERR-14 Errores de presupuesto y cálculo</t>
+          <t>ERR-13 Errores de roles y responsabilidades</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
         <is>
-          <t>Horas hombre en relación a Tareas: Fórmula =MULTIPLY inexistente en Excel (#¿NOMBRE?) y totales escritos a mano.</t>
+          <t>Matriz RACI: La misma persona era Responsable (R) y Aprobador (A) en Desarrollo de la Aplicación de Escritorio.</t>
         </is>
       </c>
       <c r="E215" s="2" t="inlineStr">
         <is>
-          <t>Fuente B: bloque ERR-14 · Fuente A: AUDIT-075, párrafo P277 (Horas hombre en relación a Tareas.xlsx (1.6))</t>
+          <t>Fuente B: bloque ERR-13 · Fuente A: AUDIT-069, párrafo P251 (Matriz RACI.xlsx (1.5))</t>
         </is>
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>Ausente (incorporado el 17/10/2026)</t>
+          <t>Ausente</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
         <is>
-          <t>Ausente</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="H215" s="2" t="inlineStr">
         <is>
-          <t>Horas hombre: F10:F36 = E*C (sin MULTIPLY); C38 =SUM(C10:C36) = 88 h; F38 =SUM(F10:F36) = $1.032.000. Comprobado por recálculo en Python sobre el detalle.</t>
-        </is>
-      </c>
-      <c r="I215" s="4" t="inlineStr">
+          <t>Matriz RACI: filas 10, 11, 2-3 y 14 según lo indicado</t>
+        </is>
+      </c>
+      <c r="I215" s="3" t="inlineStr">
         <is>
           <t>Verificado</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde parcial</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr">
         <is>
-          <t>verde</t>
+          <t>verde parcial</t>
         </is>
       </c>
       <c r="L215" s="2" t="inlineStr">
         <is>
-          <t>Corregido el 18/10/2026: fórmulas =E*C y totales =SUM. Causa raíz confirmada: MULTIPLY no existe en Excel y los totales estaban escritos a mano. Archivo: Horas hombre en relación a Tareas.xlsx. Limitación: no abierto en Excel para ver el recálculo.</t>
+          <t>Mantener (verde correcto)</t>
         </is>
       </c>
     </row>
     <row r="216" ht="45" customHeight="1">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>[ERR-14.03]</t>
+          <t>[ERR-13.05]</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>AUDIT-076</t>
+          <t>AUDIT-070</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>ERR-14 Errores de presupuesto y cálculo</t>
+          <t>ERR-13 Errores de roles y responsabilidades</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>Horas hombre en relación a Tareas: Resumen por responsable con las horas y montos de Gabriel y Alonso intercambiados.</t>
+          <t>Matriz RACI: La misma persona era R y A en Testing QA, y el Product Owner solo figuraba como Informado.</t>
         </is>
       </c>
       <c r="E216" s="2" t="inlineStr">
         <is>
-          <t>Fuente B: bloque ERR-14 · Fuente A: AUDIT-076, párrafo P281 (Horas hombre en relación a Tareas.xlsx (1.6))</t>
+          <t>Fuente B: bloque ERR-13 · Fuente A: AUDIT-070, párrafo P255 (Matriz RACI.xlsx (1.5))</t>
         </is>
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>Ausente (incorporado el 17/10/2026)</t>
+          <t>Ausente</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
         <is>
-          <t>Ausente</t>
+          <t>Presente</t>
         </is>
       </c>
       <c r="H216" s="2" t="inlineStr">
         <is>
-          <t>Horas hombre: resumen con SUMIF: Gabriel 12 h/$120.000; Diego 47 h/$564.000; Alonso 29 h/$348.000 (criterio 'Alonso*'). Comprobado por recálculo: coincide con el detalle.</t>
-        </is>
-      </c>
-      <c r="I216" s="4" t="inlineStr">
+          <t>Matriz RACI: filas 10, 11, 2-3 y 14 según lo indicado</t>
+        </is>
+      </c>
+      <c r="I216" s="3" t="inlineStr">
         <is>
           <t>Verificado</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde parcial</t>
         </is>
       </c>
       <c r="K216" s="2" t="inlineStr">
         <is>
-          <t>verde</t>
+          <t>verde parcial</t>
         </is>
       </c>
       <c r="L216" s="2" t="inlineStr">
         <is>
-          <t>Corregido el 18/10/2026: resumen por responsable con SUMIF sobre la columna D. Causa raíz confirmada: valores fijos intercambiados entre Gabriel y Alonso. Riesgo evitado: «Alonso Gonzalez» (sin tilde) en el detalle; con coincidencia exacta el SUMIF daría 0. Archivo: Horas hombre en relación a Tareas.xlsx.</t>
+          <t>Mantener (verde correcto)</t>
         </is>
       </c>
     </row>
     <row r="217" ht="90" customHeight="1">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>[ERR-15.01]</t>
+          <t>[ERR-13.06]</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>AUDIT-008, AUDIT-P13</t>
+          <t>AUDIT-071</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>ERR-15 Errores de control documental (versiones, índices, anexos y diagramas)</t>
+          <t>ERR-13 Errores de roles y responsabilidades</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>Bitácora de cambios (Hoja de ruta): Entrada '(07/10/2026)' registrada sin texto en la bitácora.</t>
+          <t>Matriz RACI: El Product Owner figuraba solo como Informado, incluso en Definición de requisitos.</t>
         </is>
       </c>
       <c r="E217" s="2" t="inlineStr">
         <is>
-          <t>Fuente B: bloque ERR-15 · Fuente A: AUDIT-008, párrafo P16 (1.2.1 Hoja de ruta del proyecto)</t>
+          <t>Fuente B: bloque ERR-13 · Fuente A: AUDIT-071, párrafo P259 (Matriz RACI.xlsx (1.5))</t>
         </is>
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
+          <t>Ausente</t>
+        </is>
+      </c>
+      <c r="G217" s="2" t="inlineStr">
+        <is>
           <t>Presente</t>
         </is>
       </c>
-      <c r="G217" s="2" t="inlineStr">
-        <is>
-          <t>Ausente</t>
-        </is>
-      </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
-          <t>Entrada vacía solo existe en la copia de referencia (AUDITORIA CLAUDE); Cambios Realizados.docx actual ya no la contiene</t>
-        </is>
-      </c>
-      <c r="I217" s="6" t="inlineStr">
-        <is>
-          <t>No determinable</t>
+          <t>Matriz RACI: filas 10, 11, 2-3 y 14 según lo indicado</t>
+        </is>
+      </c>
+      <c r="I217" s="3" t="inlineStr">
+        <is>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde parcial</t>
         </is>
       </c>
       <c r="K217" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde parcial</t>
         </is>
       </c>
       <c r="L217" s="2" t="inlineStr">
         <is>
-          <t>Investigar (no determinable con los archivos)</t>
+          <t>Mantener (verde correcto)</t>
         </is>
       </c>
     </row>
     <row r="218" ht="90" customHeight="1">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>[ERR-15.02]</t>
+          <t>[ERR-13.07]</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t>AUDIT-052</t>
+          <t>AUDIT-072</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>ERR-15 Errores de control documental (versiones, índices, anexos y diagramas)</t>
+          <t>ERR-13 Errores de roles y responsabilidades</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>Acta de constitución: Control de cambios sin la versión vigente con fecha real (faltaba la v1.2).</t>
+          <t>Matriz RACI: Faltaba la actividad 'Aceptación de incrementos (Sprint Review)' exigida por el Plan de pruebas.</t>
         </is>
       </c>
       <c r="E218" s="2" t="inlineStr">
         <is>
-          <t>Fuente B: bloque ERR-15 · Fuente A: AUDIT-052, párrafo P181 (Acta de constitución.docx (1.3))</t>
+          <t>Fuente B: bloque ERR-13 · Fuente A: AUDIT-072, párrafo P263 (Matriz RACI.xlsx (1.5))</t>
         </is>
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
+          <t>Ausente</t>
+        </is>
+      </c>
+      <c r="G218" s="2" t="inlineStr">
+        <is>
           <t>Presente</t>
         </is>
       </c>
-      <c r="G218" s="2" t="inlineStr">
-        <is>
-          <t>Presente</t>
-        </is>
-      </c>
       <c r="H218" s="2" t="inlineStr">
         <is>
-          <t>Acta: control de cambios v1.2 Gabriel Valencia 07-10-2026</t>
+          <t>Matriz RACI: filas 10, 11, 2-3 y 14 según lo indicado</t>
         </is>
       </c>
       <c r="I218" s="3" t="inlineStr">
@@ -13997,42 +13997,42 @@
     <row r="219" ht="90" customHeight="1">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>[ERR-15.03]</t>
+          <t>[ERR-13.08]</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
         <is>
-          <t>AUDIT-054</t>
+          <t>AUDIT-112</t>
         </is>
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>ERR-15 Errores de control documental (versiones, índices, anexos y diagramas)</t>
+          <t>ERR-13 Errores de roles y responsabilidades</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
         <is>
-          <t>Informe ERS: Ficha del documento con una sola revisión (v1.0); no había historial de versiones.</t>
+          <t>2.1.1 PRODUCT BACKLOG: Se mencionaban 'dos Developers' cuando el equipo tiene tres integrantes con tareas de desarrollo.</t>
         </is>
       </c>
       <c r="E219" s="2" t="inlineStr">
         <is>
-          <t>Fuente B: bloque ERR-15 · Fuente A: AUDIT-054, párrafo P190 (Informe ERS.docx (1.4))</t>
+          <t>Fuente B: bloque ERR-13 · Fuente A: AUDIT-112, párrafo P426 (2.1.1 PRODUCT BACKLOG.docx (2.1))</t>
         </is>
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
+          <t>Ausente</t>
+        </is>
+      </c>
+      <c r="G219" s="2" t="inlineStr">
+        <is>
           <t>Presente</t>
         </is>
       </c>
-      <c r="G219" s="2" t="inlineStr">
-        <is>
-          <t>Presente</t>
-        </is>
-      </c>
       <c r="H219" s="2" t="inlineStr">
         <is>
-          <t>ERS: ficha con revisión 1.1 (07/10/2026, Gabriel Valencia)</t>
+          <t>Product Backlog §10: "tres Developers"</t>
         </is>
       </c>
       <c r="I219" s="3" t="inlineStr">
@@ -14059,94 +14059,94 @@
     <row r="220" ht="90" customHeight="1">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>[ERR-15.04]</t>
+          <t>[ERR-13.09]</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
         <is>
-          <t>AUDIT-067</t>
+          <t>AUDIT-P09</t>
         </is>
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>ERR-15 Errores de control documental (versiones, índices, anexos y diagramas)</t>
+          <t>ERR-13 Errores de roles y responsabilidades</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t>Informe ERS: Anexo 'Carta Gantt' sin contenido.</t>
+          <t>[Pendiente] Cambios Pendientes: El rebalanceo de la carga de Alonso (BD, web y móvil) en la RACI sigue sin resolverse.</t>
         </is>
       </c>
       <c r="E220" s="2" t="inlineStr">
         <is>
-          <t>Fuente B: bloque ERR-15 · Fuente A: AUDIT-067, párrafo P242 (Informe ERS.docx (1.4))</t>
+          <t>Fuente B: bloque ERR-13</t>
         </is>
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="G220" s="2" t="inlineStr">
+        <is>
           <t>Ausente</t>
         </is>
       </c>
-      <c r="G220" s="2" t="inlineStr">
-        <is>
-          <t>Presente</t>
-        </is>
-      </c>
       <c r="H220" s="2" t="inlineStr">
         <is>
-          <t>ERS Anexo Carta Gantt: texto nuevo literal</t>
-        </is>
-      </c>
-      <c r="I220" s="3" t="inlineStr">
-        <is>
-          <t>Verificado</t>
+          <t>Ítem de Cambios Pendientes</t>
+        </is>
+      </c>
+      <c r="I220" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente (AUDIT-P09)</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>verde parcial</t>
+          <t>sin resaltar</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr">
         <is>
-          <t>verde parcial</t>
+          <t>sin resaltar</t>
         </is>
       </c>
       <c r="L220" s="2" t="inlineStr">
         <is>
-          <t>Mantener (verde correcto)</t>
+          <t>Mantener en Cambios Pendientes</t>
         </is>
       </c>
     </row>
     <row r="221" ht="90" customHeight="1">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>[ERR-15.05]</t>
+          <t>[ERR-14.01]</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
         <is>
-          <t>AUDIT-068</t>
+          <t>AUDIT-073</t>
         </is>
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>ERR-15 Errores de control documental (versiones, índices, anexos y diagramas)</t>
+          <t>ERR-14 Errores de presupuesto y cálculo</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>Informe ERS: El índice duplicaba 'Limitaciones', omitía la sección 2.3 y rotulaba mal el anexo.</t>
+          <t>Informe TEC: El índice anunciaba la sección de Presupuesto de Infraestructura, pero no existía (faltaban costos de SMS, hosting, Maps y tiendas).</t>
         </is>
       </c>
       <c r="E221" s="2" t="inlineStr">
         <is>
-          <t>Fuente B: bloque ERR-15 · Fuente A: AUDIT-068, párrafo P246 (Informe ERS.docx (1.4))</t>
+          <t>Fuente B: bloque ERR-14 · Fuente A: AUDIT-073, párrafo P268 (Informe TEC.docx (1.6))</t>
         </is>
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>Presente</t>
+          <t>Ausente (incorporado el 17/10/2026)</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -14156,12 +14156,12 @@
       </c>
       <c r="H221" s="2" t="inlineStr">
         <is>
-          <t>ERS índice: ya no repite Limitaciones e incluye Hitos (numerado 3.); el anexo remite a "sección 2.3"; páginas sin validar</t>
-        </is>
-      </c>
-      <c r="I221" s="5" t="inlineStr">
-        <is>
-          <t>Parcial</t>
+          <t>Informe TEC: sección «Presupuesto de Infraestructura y Herramientas a Utilizar» presente entre «Tarifas» y «Resumen Financiero»; el índice enlaza a ella (marcador _9m3x90b8fdyy). Total $1.496.400 sin cambios.</t>
+        </is>
+      </c>
+      <c r="I221" s="4" t="inlineStr">
+        <is>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J221" s="2" t="inlineStr">
@@ -14171,59 +14171,59 @@
       </c>
       <c r="K221" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="L221" s="2" t="inlineStr">
         <is>
-          <t>Investigar / mantener pendiente (corrección parcial)</t>
+          <t>Corregido el 18/10/2026: sección creada con costos conocidos ($0 en herramientas, PayPal sandbox, Firebase, Maps, jsReport, Mindicador) y pendientes marcados (mensajería, hosting, tiendas). Causa raíz confirmada: sección inexistente. Archivo: Informe TEC.docx. Limitación: páginas del índice sin actualizar (hacerlo en Word); no abierto en Word para revisión visual.</t>
         </is>
       </c>
     </row>
     <row r="222" ht="90" customHeight="1">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>[ERR-15.06]</t>
+          <t>[ERR-14.02]</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>AUDIT-157</t>
+          <t>AUDIT-075</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>ERR-15 Errores de control documental (versiones, índices, anexos y diagramas)</t>
+          <t>ERR-14 Errores de presupuesto y cálculo</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>Plan de pruebas: Control del documento solo con la versión 1.0, sin historial de versiones con fechas reales.</t>
+          <t>Horas hombre en relación a Tareas: Fórmula =MULTIPLY inexistente en Excel (#¿NOMBRE?) y totales escritos a mano.</t>
         </is>
       </c>
       <c r="E222" s="2" t="inlineStr">
         <is>
-          <t>Fuente B: bloque ERR-15 · Fuente A: AUDIT-157, párrafo P612 (Plan de pruebas.docx (2.3))</t>
+          <t>Fuente B: bloque ERR-14 · Fuente A: AUDIT-075, párrafo P277 (Horas hombre en relación a Tareas.xlsx (1.6))</t>
         </is>
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>Presente</t>
+          <t>Ausente (incorporado el 17/10/2026)</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
         <is>
-          <t>Presente</t>
+          <t>Ausente</t>
         </is>
       </c>
       <c r="H222" s="2" t="inlineStr">
         <is>
-          <t>Plan de pruebas: versión 1.1 agregada; estado "[pendiente de confirmar]"</t>
-        </is>
-      </c>
-      <c r="I222" s="5" t="inlineStr">
-        <is>
-          <t>Parcial</t>
+          <t>Horas hombre: F10:F36 = E*C (sin MULTIPLY); C38 =SUM(C10:C36) = 88 h; F38 =SUM(F10:F36) = $1.032.000. Comprobado por recálculo en Python sobre el detalle.</t>
+        </is>
+      </c>
+      <c r="I222" s="4" t="inlineStr">
+        <is>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J222" s="2" t="inlineStr">
@@ -14233,44 +14233,44 @@
       </c>
       <c r="K222" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="L222" s="2" t="inlineStr">
         <is>
-          <t>Investigar / mantener pendiente (corrección parcial)</t>
+          <t>Corregido el 18/10/2026: fórmulas =E*C y totales =SUM. Causa raíz confirmada: MULTIPLY no existe en Excel y los totales estaban escritos a mano. Archivo: Horas hombre en relación a Tareas.xlsx. Limitación: no abierto en Excel para ver el recálculo.</t>
         </is>
       </c>
     </row>
     <row r="223" ht="90" customHeight="1">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>[ERR-15.07]</t>
+          <t>[ERR-14.03]</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
         <is>
-          <t>AUDIT-P11</t>
+          <t>AUDIT-076</t>
         </is>
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>ERR-15 Errores de control documental (versiones, índices, anexos y diagramas)</t>
+          <t>ERR-14 Errores de presupuesto y cálculo</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>[Pendiente] Cambios Pendientes: Diagramas ER y de secuencia 'Generar Alerta' no actualizados con las tablas, columnas y estados nuevos.</t>
+          <t>Horas hombre en relación a Tareas: Resumen por responsable con las horas y montos de Gabriel y Alonso intercambiados.</t>
         </is>
       </c>
       <c r="E223" s="2" t="inlineStr">
         <is>
-          <t>Fuente B: bloque ERR-15</t>
+          <t>Fuente B: bloque ERR-14 · Fuente A: AUDIT-076, párrafo P281 (Horas hombre en relación a Tareas.xlsx (1.6))</t>
         </is>
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>Presente</t>
+          <t>Ausente (incorporado el 17/10/2026)</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -14280,12 +14280,12 @@
       </c>
       <c r="H223" s="2" t="inlineStr">
         <is>
-          <t>Ítem de Cambios Pendientes</t>
-        </is>
-      </c>
-      <c r="I223" s="2" t="inlineStr">
-        <is>
-          <t>Pendiente (AUDIT-P11)</t>
+          <t>Horas hombre: resumen con SUMIF: Gabriel 12 h/$120.000; Diego 47 h/$564.000; Alonso 29 h/$348.000 (criterio 'Alonso*'). Comprobado por recálculo: coincide con el detalle.</t>
+        </is>
+      </c>
+      <c r="I223" s="4" t="inlineStr">
+        <is>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr">
@@ -14295,134 +14295,568 @@
       </c>
       <c r="K223" s="2" t="inlineStr">
         <is>
-          <t>sin resaltar</t>
+          <t>verde</t>
         </is>
       </c>
       <c r="L223" s="2" t="inlineStr">
         <is>
-          <t>Mantener en Cambios Pendientes</t>
+          <t>Corregido el 18/10/2026: resumen por responsable con SUMIF sobre la columna D. Causa raíz confirmada: valores fijos intercambiados entre Gabriel y Alonso. Riesgo evitado: «Alonso Gonzalez» (sin tilde) en el detalle; con coincidencia exacta el SUMIF daría 0. Archivo: Horas hombre en relación a Tareas.xlsx.</t>
         </is>
       </c>
     </row>
     <row r="224" ht="60" customHeight="1">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>[ERR-16.01]</t>
+          <t>[ERR-15.01]</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
         <is>
-          <t>AUDIT-039</t>
+          <t>AUDIT-008, AUDIT-P13</t>
         </is>
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>ERR-16 Referencias a normas y estándares obsoletos</t>
+          <t>ERR-15 Errores de control documental (versiones, índices, anexos y diagramas)</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>Acta de constitución: Se exigía cumplir ISO 9126 (reemplazada por ISO/IEC 25010) e ISO 25001 (que no es un modelo de calidad de producto).</t>
+          <t>Bitácora de cambios (Hoja de ruta): Entrada '(07/10/2026)' registrada sin texto en la bitácora.</t>
         </is>
       </c>
       <c r="E224" s="2" t="inlineStr">
         <is>
-          <t>Fuente B: bloque ERR-16 · Fuente A: AUDIT-039, párrafo P129 (Acta de constitución.docx (1.3))</t>
+          <t>Fuente B: bloque ERR-15 · Fuente A: AUDIT-008, párrafo P16 (1.2.1 Hoja de ruta del proyecto)</t>
         </is>
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="G224" s="2" t="inlineStr">
+        <is>
           <t>Ausente</t>
         </is>
       </c>
-      <c r="G224" s="2" t="inlineStr">
-        <is>
-          <t>Presente</t>
-        </is>
-      </c>
       <c r="H224" s="2" t="inlineStr">
         <is>
-          <t>Acta: "modelo de calidad de producto ISO/IEC 25010"</t>
-        </is>
-      </c>
-      <c r="I224" s="3" t="inlineStr">
-        <is>
-          <t>Verificado</t>
+          <t>Entrada vacía solo existe en la copia de referencia (AUDITORIA CLAUDE); Cambios Realizados.docx actual ya no la contiene</t>
+        </is>
+      </c>
+      <c r="I224" s="6" t="inlineStr">
+        <is>
+          <t>No determinable</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>verde parcial</t>
+          <t>sin resaltar</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr">
         <is>
-          <t>verde parcial</t>
+          <t>sin resaltar</t>
         </is>
       </c>
       <c r="L224" s="2" t="inlineStr">
         <is>
-          <t>Mantener (verde correcto)</t>
+          <t>Investigar (no determinable con los archivos)</t>
         </is>
       </c>
     </row>
     <row r="225" ht="60" customHeight="1">
       <c r="A225" s="2" t="inlineStr">
         <is>
+          <t>[ERR-15.02]</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>AUDIT-052</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>ERR-15 Errores de control documental (versiones, índices, anexos y diagramas)</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>Acta de constitución: Control de cambios sin la versión vigente con fecha real (faltaba la v1.2).</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="inlineStr">
+        <is>
+          <t>Fuente B: bloque ERR-15 · Fuente A: AUDIT-052, párrafo P181 (Acta de constitución.docx (1.3))</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="G225" s="2" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="H225" s="2" t="inlineStr">
+        <is>
+          <t>Acta: control de cambios v1.2 Gabriel Valencia 07-10-2026</t>
+        </is>
+      </c>
+      <c r="I225" s="3" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="J225" s="2" t="inlineStr">
+        <is>
+          <t>verde parcial</t>
+        </is>
+      </c>
+      <c r="K225" s="2" t="inlineStr">
+        <is>
+          <t>verde parcial</t>
+        </is>
+      </c>
+      <c r="L225" s="2" t="inlineStr">
+        <is>
+          <t>Mantener (verde correcto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>[ERR-15.03]</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>AUDIT-054</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>ERR-15 Errores de control documental (versiones, índices, anexos y diagramas)</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>Informe ERS: Ficha del documento con una sola revisión (v1.0); no había historial de versiones.</t>
+        </is>
+      </c>
+      <c r="E226" s="2" t="inlineStr">
+        <is>
+          <t>Fuente B: bloque ERR-15 · Fuente A: AUDIT-054, párrafo P190 (Informe ERS.docx (1.4))</t>
+        </is>
+      </c>
+      <c r="F226" s="2" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="G226" s="2" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="H226" s="2" t="inlineStr">
+        <is>
+          <t>ERS: ficha con revisión 1.1 (07/10/2026, Gabriel Valencia)</t>
+        </is>
+      </c>
+      <c r="I226" s="3" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="J226" s="2" t="inlineStr">
+        <is>
+          <t>verde parcial</t>
+        </is>
+      </c>
+      <c r="K226" s="2" t="inlineStr">
+        <is>
+          <t>verde parcial</t>
+        </is>
+      </c>
+      <c r="L226" s="2" t="inlineStr">
+        <is>
+          <t>Mantener (verde correcto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>[ERR-15.04]</t>
+        </is>
+      </c>
+      <c r="B227" s="2" t="inlineStr">
+        <is>
+          <t>AUDIT-067</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="inlineStr">
+        <is>
+          <t>ERR-15 Errores de control documental (versiones, índices, anexos y diagramas)</t>
+        </is>
+      </c>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>Informe ERS: Anexo 'Carta Gantt' sin contenido.</t>
+        </is>
+      </c>
+      <c r="E227" s="2" t="inlineStr">
+        <is>
+          <t>Fuente B: bloque ERR-15 · Fuente A: AUDIT-067, párrafo P242 (Informe ERS.docx (1.4))</t>
+        </is>
+      </c>
+      <c r="F227" s="2" t="inlineStr">
+        <is>
+          <t>Ausente</t>
+        </is>
+      </c>
+      <c r="G227" s="2" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="H227" s="2" t="inlineStr">
+        <is>
+          <t>ERS Anexo Carta Gantt: texto nuevo literal</t>
+        </is>
+      </c>
+      <c r="I227" s="3" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="J227" s="2" t="inlineStr">
+        <is>
+          <t>verde parcial</t>
+        </is>
+      </c>
+      <c r="K227" s="2" t="inlineStr">
+        <is>
+          <t>verde parcial</t>
+        </is>
+      </c>
+      <c r="L227" s="2" t="inlineStr">
+        <is>
+          <t>Mantener (verde correcto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>[ERR-15.05]</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
+        <is>
+          <t>AUDIT-068</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="inlineStr">
+        <is>
+          <t>ERR-15 Errores de control documental (versiones, índices, anexos y diagramas)</t>
+        </is>
+      </c>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>Informe ERS: El índice duplicaba 'Limitaciones', omitía la sección 2.3 y rotulaba mal el anexo.</t>
+        </is>
+      </c>
+      <c r="E228" s="2" t="inlineStr">
+        <is>
+          <t>Fuente B: bloque ERR-15 · Fuente A: AUDIT-068, párrafo P246 (Informe ERS.docx (1.4))</t>
+        </is>
+      </c>
+      <c r="F228" s="2" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="G228" s="2" t="inlineStr">
+        <is>
+          <t>Ausente</t>
+        </is>
+      </c>
+      <c r="H228" s="2" t="inlineStr">
+        <is>
+          <t>ERS índice: ya no repite Limitaciones e incluye Hitos (numerado 3.); el anexo remite a "sección 2.3"; páginas sin validar</t>
+        </is>
+      </c>
+      <c r="I228" s="5" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="J228" s="2" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="K228" s="2" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="L228" s="2" t="inlineStr">
+        <is>
+          <t>Investigar / mantener pendiente (corrección parcial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>[ERR-15.06]</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>AUDIT-157</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr">
+        <is>
+          <t>ERR-15 Errores de control documental (versiones, índices, anexos y diagramas)</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>Plan de pruebas: Control del documento solo con la versión 1.0, sin historial de versiones con fechas reales.</t>
+        </is>
+      </c>
+      <c r="E229" s="2" t="inlineStr">
+        <is>
+          <t>Fuente B: bloque ERR-15 · Fuente A: AUDIT-157, párrafo P612 (Plan de pruebas.docx (2.3))</t>
+        </is>
+      </c>
+      <c r="F229" s="2" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="G229" s="2" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="H229" s="2" t="inlineStr">
+        <is>
+          <t>Plan de pruebas: versión 1.1 agregada; estado "[pendiente de confirmar]"</t>
+        </is>
+      </c>
+      <c r="I229" s="5" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="J229" s="2" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="K229" s="2" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="L229" s="2" t="inlineStr">
+        <is>
+          <t>Investigar / mantener pendiente (corrección parcial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>[ERR-15.07]</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>AUDIT-P11</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="inlineStr">
+        <is>
+          <t>ERR-15 Errores de control documental (versiones, índices, anexos y diagramas)</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>[Pendiente] Cambios Pendientes: Diagramas ER y de secuencia 'Generar Alerta' no actualizados con las tablas, columnas y estados nuevos.</t>
+        </is>
+      </c>
+      <c r="E230" s="2" t="inlineStr">
+        <is>
+          <t>Fuente B: bloque ERR-15</t>
+        </is>
+      </c>
+      <c r="F230" s="2" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="G230" s="2" t="inlineStr">
+        <is>
+          <t>Ausente</t>
+        </is>
+      </c>
+      <c r="H230" s="2" t="inlineStr">
+        <is>
+          <t>Ítem de Cambios Pendientes</t>
+        </is>
+      </c>
+      <c r="I230" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente (AUDIT-P11)</t>
+        </is>
+      </c>
+      <c r="J230" s="2" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="K230" s="2" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="L230" s="2" t="inlineStr">
+        <is>
+          <t>Mantener en Cambios Pendientes</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>[ERR-16.01]</t>
+        </is>
+      </c>
+      <c r="B231" s="2" t="inlineStr">
+        <is>
+          <t>AUDIT-039</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="inlineStr">
+        <is>
+          <t>ERR-16 Referencias a normas y estándares obsoletos</t>
+        </is>
+      </c>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>Acta de constitución: Se exigía cumplir ISO 9126 (reemplazada por ISO/IEC 25010) e ISO 25001 (que no es un modelo de calidad de producto).</t>
+        </is>
+      </c>
+      <c r="E231" s="2" t="inlineStr">
+        <is>
+          <t>Fuente B: bloque ERR-16 · Fuente A: AUDIT-039, párrafo P129 (Acta de constitución.docx (1.3))</t>
+        </is>
+      </c>
+      <c r="F231" s="2" t="inlineStr">
+        <is>
+          <t>Ausente</t>
+        </is>
+      </c>
+      <c r="G231" s="2" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="H231" s="2" t="inlineStr">
+        <is>
+          <t>Acta: "modelo de calidad de producto ISO/IEC 25010"</t>
+        </is>
+      </c>
+      <c r="I231" s="3" t="inlineStr">
+        <is>
+          <t>Verificado</t>
+        </is>
+      </c>
+      <c r="J231" s="2" t="inlineStr">
+        <is>
+          <t>verde parcial</t>
+        </is>
+      </c>
+      <c r="K231" s="2" t="inlineStr">
+        <is>
+          <t>verde parcial</t>
+        </is>
+      </c>
+      <c r="L231" s="2" t="inlineStr">
+        <is>
+          <t>Mantener (verde correcto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
           <t>[ERR-16.02]</t>
         </is>
       </c>
-      <c r="B225" s="2" t="inlineStr">
+      <c r="B232" s="2" t="inlineStr">
         <is>
           <t>AUDIT-053</t>
         </is>
       </c>
-      <c r="C225" s="2" t="inlineStr">
+      <c r="C232" s="2" t="inlineStr">
         <is>
           <t>ERR-16 Referencias a normas y estándares obsoletos</t>
         </is>
       </c>
-      <c r="D225" s="2" t="inlineStr">
+      <c r="D232" s="2" t="inlineStr">
         <is>
           <t>Informe ERS: Se citaba IEEE 830, reemplazada por ISO/IEC/IEEE 29148:2018.</t>
         </is>
       </c>
-      <c r="E225" s="2" t="inlineStr">
+      <c r="E232" s="2" t="inlineStr">
         <is>
           <t>Fuente B: bloque ERR-16 · Fuente A: AUDIT-053, párrafo P186 (Informe ERS.docx (1.4))</t>
         </is>
       </c>
-      <c r="F225" s="2" t="inlineStr">
+      <c r="F232" s="2" t="inlineStr">
         <is>
           <t>Presente</t>
         </is>
       </c>
-      <c r="G225" s="2" t="inlineStr">
+      <c r="G232" s="2" t="inlineStr">
         <is>
           <t>Presente</t>
         </is>
       </c>
-      <c r="H225" s="2" t="inlineStr">
+      <c r="H232" s="2" t="inlineStr">
         <is>
           <t>ERS: no aparece la frase de portada ni IEEE 830 ni ISO/IEC/IEEE 29148</t>
         </is>
       </c>
-      <c r="I225" s="6" t="inlineStr">
+      <c r="I232" s="6" t="inlineStr">
         <is>
           <t>No determinable</t>
         </is>
       </c>
-      <c r="J225" s="2" t="inlineStr">
-        <is>
-          <t>sin resaltar</t>
-        </is>
-      </c>
-      <c r="K225" s="2" t="inlineStr">
-        <is>
-          <t>sin resaltar</t>
-        </is>
-      </c>
-      <c r="L225" s="2" t="inlineStr">
+      <c r="J232" s="2" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="K232" s="2" t="inlineStr">
+        <is>
+          <t>sin resaltar</t>
+        </is>
+      </c>
+      <c r="L232" s="2" t="inlineStr">
         <is>
           <t>Investigar (no determinable con los archivos)</t>
         </is>
@@ -15509,12 +15943,12 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Hoja de ruta §7: "horizonte claro de 7 semanas"</t>
+          <t>Hoja de ruta §7: horizonte de 5 semanas (verificado 18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -15593,12 +16027,12 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Hoja de ruta: no existe la "Nota de fechas"</t>
+          <t>Hoja de ruta §7: nota de fechas añadida (verificado 18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -15635,12 +16069,12 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Hoja de ruta §6: siguen dos listas de DoD</t>
+          <t>Hoja de ruta §6: DoD única de 8 ítems (verificado 18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -15677,12 +16111,12 @@
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Sprint-fase1: PBI siguen como F1-01…F1-11</t>
+          <t>Sprint-fase1: TD-01…TD-11 (verificado 18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -17118,7 +17552,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>ERS: no existe la nota de conciliación por plataforma</t>
+          <t>Pendiente: nota de planificación por HU en el ERS sin aprobar (18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -17569,12 +18003,12 @@
       <c r="F79" s="2" t="n"/>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>Product Backlog §3: "10 de agosto al 6 de septiembre"</t>
+          <t>Product Backlog §3 y §7: cierre 14 de septiembre (verificado 18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -18557,12 +18991,12 @@
       <c r="F105" s="2" t="n"/>
       <c r="G105" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>Product Backlog §7: "cuatro Sprints de una semana"</t>
+          <t>Product Backlog §7: cadencia corregida (verificado 18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -18633,12 +19067,12 @@
       <c r="F107" s="2" t="n"/>
       <c r="G107" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>Product Backlog §7: DoD propia de 6 ítems</t>
+          <t>Product Backlog §7: DoD remite a Hoja §6 (verificado 18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -18823,12 +19257,12 @@
       <c r="F112" s="2" t="n"/>
       <c r="G112" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>Product Backlog §8: tabla con 13 HU y sin nota de numeración</t>
+          <t>Product Backlog §8: Sprint renumerado +4 (verificado 18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -18975,12 +19409,12 @@
       <c r="F116" s="2" t="n"/>
       <c r="G116" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>Tabla Maestra sin cambios: dependencias F1-xx, features cruzadas, CA originales (CA-03.1 en C5 y CA-08.1 en C11 de la hoja "Criterio de aceptacion")</t>
+          <t>Tabla Maestra: TD-xx en dependencias (verificado 18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -19317,12 +19751,12 @@
       <c r="F125" s="2" t="n"/>
       <c r="G125" s="4" t="inlineStr">
         <is>
-          <t>No aplicado</t>
+          <t>Verificado</t>
         </is>
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>Tabla Maestra sin cambios: dependencias F1-xx, features cruzadas, CA originales (CA-03.1 en C5 y CA-08.1 en C11 de la hoja "Criterio de aceptacion")</t>
+          <t>Tabla Maestra: hoja Tareas F1 con TD-xx y prioridades (verificado 18/10/2026)</t>
         </is>
       </c>
     </row>

</xml_diff>